<commit_message>
RF05-RF06: result schema, drilldown seguro y docs
</commit_message>
<xml_diff>
--- a/requisitos_backlog.xlsx
+++ b/requisitos_backlog.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luciasorniscaletti/Desktop/UNI/TFG/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luciasorniscaletti/Desktop/UNI/TFG/erp-fraud-data-TFG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4D395C3-8C13-564B-9F64-D93D374002FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07FCA33A-A140-544F-A709-B0B43DDE0B09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3515,6 +3515,9 @@
       <c r="C78" s="20">
         <v>1.2</v>
       </c>
+      <c r="D78" s="20">
+        <v>1</v>
+      </c>
     </row>
     <row r="79" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B79" s="21" t="s">
@@ -3523,6 +3526,9 @@
       <c r="C79" s="20">
         <v>0.8</v>
       </c>
+      <c r="D79" s="20">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="80" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B80" s="21" t="s">
@@ -3531,72 +3537,96 @@
       <c r="C80" s="20">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="81" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="D80" s="20">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B81" s="21" t="s">
         <v>162</v>
       </c>
       <c r="C81" s="20">
         <v>1</v>
       </c>
-    </row>
-    <row r="82" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="D81" s="20">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B82" s="21" t="s">
         <v>163</v>
       </c>
       <c r="C82" s="20">
         <v>1.5</v>
       </c>
-    </row>
-    <row r="83" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="D82" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B83" s="21" t="s">
         <v>164</v>
       </c>
       <c r="C83" s="20">
         <v>1</v>
       </c>
-    </row>
-    <row r="84" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="D83" s="20">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B84" s="21" t="s">
         <v>165</v>
       </c>
       <c r="C84" s="20">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="85" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="D84" s="20">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B85" s="21" t="s">
         <v>166</v>
       </c>
       <c r="C85" s="20">
         <v>1.5</v>
       </c>
-    </row>
-    <row r="86" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="D85" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="B86" s="21" t="s">
         <v>167</v>
       </c>
       <c r="C86" s="20">
         <v>1</v>
       </c>
-    </row>
-    <row r="87" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="D86" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B87" s="21" t="s">
         <v>168</v>
       </c>
       <c r="C87" s="20">
         <v>1</v>
       </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D87" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B88" s="21"/>
     </row>
-    <row r="89" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:4" ht="18" x14ac:dyDescent="0.2">
       <c r="A89" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="90" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B90" s="21" t="s">
         <v>169</v>
       </c>
@@ -3604,7 +3634,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B91" s="21" t="s">
         <v>170</v>
       </c>
@@ -3612,7 +3642,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="92" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B92" s="21" t="s">
         <v>171</v>
       </c>
@@ -3620,7 +3650,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="93" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B93" s="21" t="s">
         <v>172</v>
       </c>
@@ -3628,7 +3658,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B94" s="21" t="s">
         <v>173</v>
       </c>
@@ -3636,7 +3666,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B95" s="21" t="s">
         <v>174</v>
       </c>
@@ -3644,7 +3674,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="96" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B96" s="21" t="s">
         <v>175</v>
       </c>

</xml_diff>

<commit_message>
RF07-RF10: ranking, reporting MVP, comando run y Makefile
</commit_message>
<xml_diff>
--- a/requisitos_backlog.xlsx
+++ b/requisitos_backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luciasorniscaletti/Desktop/UNI/TFG/erp-fraud-data-TFG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07FCA33A-A140-544F-A709-B0B43DDE0B09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{255D40C0-4C68-604E-91A5-A7537108CA18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -633,9 +633,6 @@
     <t>RF08-03: Implementar generador de reporte MD a partir de report.json</t>
   </si>
   <si>
-    <t>RF08-04: Implementar opcional render MD→HTML (si decides) y guardarlo en run_results</t>
-  </si>
-  <si>
     <t>RF08-05: Incluir enlaces/rutas a outputs por test y a data_dictionary/schema_summary</t>
   </si>
   <si>
@@ -1342,6 +1339,9 @@
   </si>
   <si>
     <t>AG03-04: Documentar 2–3 iteraciones reales (prompt→diff→validación) como evidencia en docs/codex_workflow.md</t>
+  </si>
+  <si>
+    <t>RF08-04: Implementar opcional render MD→HTML (si decido) y guardarlo en run_results</t>
   </si>
 </sst>
 </file>
@@ -1474,7 +1474,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1547,6 +1547,18 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1821,7 +1833,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>5</v>
@@ -1835,13 +1847,13 @@
     </row>
     <row r="2" spans="1:9" customFormat="1" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="22" t="s">
+        <v>375</v>
+      </c>
+      <c r="B2" s="23" t="s">
         <v>376</v>
       </c>
-      <c r="B2" s="23" t="s">
+      <c r="C2" s="22" t="s">
         <v>377</v>
-      </c>
-      <c r="C2" s="22" t="s">
-        <v>378</v>
       </c>
       <c r="D2">
         <v>3</v>
@@ -1855,13 +1867,13 @@
     </row>
     <row r="3" spans="1:9" customFormat="1" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="22" t="s">
+        <v>378</v>
+      </c>
+      <c r="B3" s="23" t="s">
         <v>379</v>
       </c>
-      <c r="B3" s="23" t="s">
+      <c r="C3" s="22" t="s">
         <v>380</v>
-      </c>
-      <c r="C3" s="22" t="s">
-        <v>381</v>
       </c>
       <c r="D3">
         <v>5</v>
@@ -2080,28 +2092,28 @@
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
     </row>
-    <row r="13" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A13" s="12" t="s">
+    <row r="13" spans="1:9" s="29" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A13" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="B13" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="27" t="s">
         <v>40</v>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="28">
         <v>8</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="F13" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
+      <c r="G13" s="28"/>
+      <c r="H13" s="28"/>
+      <c r="I13" s="28"/>
     </row>
     <row r="14" spans="1:9" ht="38" x14ac:dyDescent="0.2">
       <c r="A14" s="12" t="s">
@@ -2254,13 +2266,13 @@
     </row>
     <row r="21" spans="1:9" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A21" s="24" t="s">
+        <v>363</v>
+      </c>
+      <c r="B21" s="23" t="s">
         <v>364</v>
       </c>
-      <c r="B21" s="23" t="s">
+      <c r="C21" s="22" t="s">
         <v>365</v>
-      </c>
-      <c r="C21" s="22" t="s">
-        <v>366</v>
       </c>
       <c r="D21">
         <v>5</v>
@@ -2274,13 +2286,13 @@
     </row>
     <row r="22" spans="1:9" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A22" s="24" t="s">
+        <v>366</v>
+      </c>
+      <c r="B22" s="23" t="s">
         <v>367</v>
       </c>
-      <c r="B22" s="23" t="s">
+      <c r="C22" s="22" t="s">
         <v>368</v>
-      </c>
-      <c r="C22" s="22" t="s">
-        <v>369</v>
       </c>
       <c r="D22">
         <v>8</v>
@@ -2294,13 +2306,13 @@
     </row>
     <row r="23" spans="1:9" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A23" s="24" t="s">
+        <v>369</v>
+      </c>
+      <c r="B23" s="23" t="s">
         <v>370</v>
       </c>
-      <c r="B23" s="23" t="s">
+      <c r="C23" s="22" t="s">
         <v>371</v>
-      </c>
-      <c r="C23" s="22" t="s">
-        <v>372</v>
       </c>
       <c r="D23">
         <v>5</v>
@@ -2314,13 +2326,13 @@
     </row>
     <row r="24" spans="1:9" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A24" s="24" t="s">
+        <v>372</v>
+      </c>
+      <c r="B24" s="23" t="s">
         <v>373</v>
       </c>
-      <c r="B24" s="23" t="s">
+      <c r="C24" s="22" t="s">
         <v>374</v>
-      </c>
-      <c r="C24" s="22" t="s">
-        <v>375</v>
       </c>
       <c r="D24">
         <v>5</v>
@@ -2598,13 +2610,13 @@
     </row>
     <row r="37" spans="1:9" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A37" s="24" t="s">
+        <v>381</v>
+      </c>
+      <c r="B37" s="23" t="s">
         <v>382</v>
       </c>
-      <c r="B37" s="23" t="s">
+      <c r="C37" s="22" t="s">
         <v>383</v>
-      </c>
-      <c r="C37" s="22" t="s">
-        <v>384</v>
       </c>
       <c r="D37">
         <v>3</v>
@@ -2754,10 +2766,10 @@
     </row>
     <row r="3" spans="1:5" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A3" s="24" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C3" s="22">
         <v>0.6</v>
@@ -2768,7 +2780,7 @@
     <row r="4" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A4" s="24"/>
       <c r="B4" s="22" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C4" s="22">
         <v>0.8</v>
@@ -2779,7 +2791,7 @@
     <row r="5" spans="1:5" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" s="24"/>
       <c r="B5" s="22" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C5" s="22">
         <v>0.8</v>
@@ -2790,7 +2802,7 @@
     <row r="6" spans="1:5" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" s="24"/>
       <c r="B6" s="22" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C6" s="22">
         <v>0.8</v>
@@ -2801,7 +2813,7 @@
     <row r="7" spans="1:5" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" s="24"/>
       <c r="B7" s="22" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C7" s="22">
         <v>0.5</v>
@@ -2812,7 +2824,7 @@
     <row r="8" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A8" s="24"/>
       <c r="B8" s="22" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C8" s="22">
         <v>0.5</v>
@@ -2822,10 +2834,10 @@
     </row>
     <row r="9" spans="1:5" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A9" s="24" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C9" s="22">
         <v>1</v>
@@ -2836,7 +2848,7 @@
     <row r="10" spans="1:5" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A10" s="24"/>
       <c r="B10" s="22" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C10" s="22">
         <v>1</v>
@@ -2847,7 +2859,7 @@
     <row r="11" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A11" s="24"/>
       <c r="B11" s="22" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C11" s="22">
         <v>1</v>
@@ -2858,7 +2870,7 @@
     <row r="12" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A12" s="24"/>
       <c r="B12" s="22" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="C12" s="22">
         <v>1</v>
@@ -2869,7 +2881,7 @@
     <row r="13" spans="1:5" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A13" s="24"/>
       <c r="B13" s="22" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C13" s="22">
         <v>1</v>
@@ -2880,7 +2892,7 @@
     <row r="14" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A14" s="24"/>
       <c r="B14" s="22" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C14" s="22">
         <v>1.2</v>
@@ -2891,7 +2903,7 @@
     <row r="15" spans="1:5" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A15" s="24"/>
       <c r="B15" s="22" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="C15" s="22">
         <v>0.6</v>
@@ -3633,6 +3645,9 @@
       <c r="C90" s="20">
         <v>1</v>
       </c>
+      <c r="D90" s="20">
+        <v>1.2</v>
+      </c>
     </row>
     <row r="91" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B91" s="21" t="s">
@@ -3641,6 +3656,9 @@
       <c r="C91" s="20">
         <v>1.2</v>
       </c>
+      <c r="D91" s="20">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="92" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B92" s="21" t="s">
@@ -3649,6 +3667,9 @@
       <c r="C92" s="20">
         <v>0.8</v>
       </c>
+      <c r="D92" s="20">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="93" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B93" s="21" t="s">
@@ -3892,7 +3913,7 @@
     </row>
     <row r="126" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B126" s="21" t="s">
-        <v>199</v>
+        <v>435</v>
       </c>
       <c r="C126" s="20">
         <v>1</v>
@@ -3900,7 +3921,7 @@
     </row>
     <row r="127" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B127" s="21" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C127" s="20">
         <v>0.8</v>
@@ -3908,7 +3929,7 @@
     </row>
     <row r="128" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B128" s="21" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C128" s="20">
         <v>0.8</v>
@@ -3916,7 +3937,7 @@
     </row>
     <row r="129" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B129" s="21" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C129" s="20">
         <v>0.8</v>
@@ -3924,7 +3945,7 @@
     </row>
     <row r="130" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B130" s="21" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C130" s="20">
         <v>1.5</v>
@@ -3932,7 +3953,7 @@
     </row>
     <row r="131" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B131" s="21" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C131" s="20">
         <v>1</v>
@@ -3940,7 +3961,7 @@
     </row>
     <row r="132" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B132" s="21" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C132" s="20">
         <v>1</v>
@@ -3956,7 +3977,7 @@
     </row>
     <row r="135" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B135" s="21" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C135" s="20">
         <v>1.5</v>
@@ -3964,7 +3985,7 @@
     </row>
     <row r="136" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B136" s="21" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C136" s="20">
         <v>0.8</v>
@@ -3972,7 +3993,7 @@
     </row>
     <row r="137" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B137" s="21" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C137" s="20">
         <v>1.5</v>
@@ -3980,7 +4001,7 @@
     </row>
     <row r="138" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B138" s="21" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C138" s="20">
         <v>1.2</v>
@@ -3988,7 +4009,7 @@
     </row>
     <row r="139" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B139" s="21" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C139" s="20">
         <v>2</v>
@@ -3996,7 +4017,7 @@
     </row>
     <row r="140" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B140" s="21" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C140" s="20">
         <v>1.5</v>
@@ -4004,7 +4025,7 @@
     </row>
     <row r="141" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B141" s="21" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C141" s="20">
         <v>1</v>
@@ -4012,7 +4033,7 @@
     </row>
     <row r="142" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B142" s="21" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C142" s="20">
         <v>1</v>
@@ -4020,7 +4041,7 @@
     </row>
     <row r="143" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B143" s="21" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C143" s="20">
         <v>1.5</v>
@@ -4028,7 +4049,7 @@
     </row>
     <row r="144" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B144" s="21" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C144" s="20">
         <v>1</v>
@@ -4044,7 +4065,7 @@
     </row>
     <row r="147" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B147" s="21" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C147" s="20">
         <v>2</v>
@@ -4052,7 +4073,7 @@
     </row>
     <row r="148" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B148" s="21" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C148" s="20">
         <v>1.2</v>
@@ -4060,7 +4081,7 @@
     </row>
     <row r="149" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B149" s="21" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C149" s="20">
         <v>1</v>
@@ -4068,7 +4089,7 @@
     </row>
     <row r="150" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B150" s="21" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C150" s="20">
         <v>1.5</v>
@@ -4076,7 +4097,7 @@
     </row>
     <row r="151" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B151" s="21" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C151" s="20">
         <v>0.8</v>
@@ -4084,7 +4105,7 @@
     </row>
     <row r="152" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B152" s="21" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C152" s="20">
         <v>1.5</v>
@@ -4092,7 +4113,7 @@
     </row>
     <row r="153" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B153" s="21" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C153" s="20">
         <v>1</v>
@@ -4100,7 +4121,7 @@
     </row>
     <row r="154" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B154" s="21" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C154" s="20">
         <v>1</v>
@@ -4116,7 +4137,7 @@
     </row>
     <row r="157" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B157" s="21" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C157" s="20">
         <v>1.5</v>
@@ -4124,7 +4145,7 @@
     </row>
     <row r="158" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B158" s="21" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C158" s="20">
         <v>1.2</v>
@@ -4132,7 +4153,7 @@
     </row>
     <row r="159" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B159" s="21" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C159" s="20">
         <v>1.5</v>
@@ -4140,7 +4161,7 @@
     </row>
     <row r="160" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B160" s="21" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C160" s="20">
         <v>2</v>
@@ -4148,7 +4169,7 @@
     </row>
     <row r="161" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B161" s="21" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C161" s="20">
         <v>1.5</v>
@@ -4156,7 +4177,7 @@
     </row>
     <row r="162" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B162" s="21" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C162" s="20">
         <v>1.5</v>
@@ -4164,7 +4185,7 @@
     </row>
     <row r="163" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B163" s="21" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C163" s="20">
         <v>1.5</v>
@@ -4172,7 +4193,7 @@
     </row>
     <row r="164" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B164" s="21" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C164" s="20">
         <v>1</v>
@@ -4180,7 +4201,7 @@
     </row>
     <row r="165" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B165" s="21" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C165" s="20">
         <v>1</v>
@@ -4196,7 +4217,7 @@
     </row>
     <row r="168" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B168" s="21" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C168" s="20">
         <v>1.2</v>
@@ -4204,7 +4225,7 @@
     </row>
     <row r="169" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B169" s="21" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C169" s="20">
         <v>1.5</v>
@@ -4212,7 +4233,7 @@
     </row>
     <row r="170" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B170" s="21" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C170" s="20">
         <v>2</v>
@@ -4220,7 +4241,7 @@
     </row>
     <row r="171" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B171" s="21" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C171" s="20">
         <v>1</v>
@@ -4228,7 +4249,7 @@
     </row>
     <row r="172" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B172" s="21" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C172" s="20">
         <v>1.2</v>
@@ -4236,7 +4257,7 @@
     </row>
     <row r="173" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B173" s="21" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C173" s="20">
         <v>1.5</v>
@@ -4244,7 +4265,7 @@
     </row>
     <row r="174" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B174" s="21" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C174" s="20">
         <v>1</v>
@@ -4252,7 +4273,7 @@
     </row>
     <row r="175" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B175" s="21" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C175" s="20">
         <v>1</v>
@@ -4268,7 +4289,7 @@
     </row>
     <row r="178" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B178" s="21" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C178" s="20">
         <v>1.5</v>
@@ -4276,7 +4297,7 @@
     </row>
     <row r="179" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B179" s="21" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C179" s="20">
         <v>0.6</v>
@@ -4284,7 +4305,7 @@
     </row>
     <row r="180" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B180" s="21" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C180" s="20">
         <v>1.2</v>
@@ -4292,7 +4313,7 @@
     </row>
     <row r="181" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B181" s="21" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C181" s="20">
         <v>0.6</v>
@@ -4300,7 +4321,7 @@
     </row>
     <row r="182" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B182" s="21" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C182" s="20">
         <v>1.2</v>
@@ -4308,7 +4329,7 @@
     </row>
     <row r="183" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B183" s="21" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C183" s="20">
         <v>2</v>
@@ -4316,7 +4337,7 @@
     </row>
     <row r="184" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B184" s="21" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C184" s="20">
         <v>1.5</v>
@@ -4324,7 +4345,7 @@
     </row>
     <row r="185" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B185" s="21" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C185" s="20">
         <v>1</v>
@@ -4332,7 +4353,7 @@
     </row>
     <row r="186" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B186" s="21" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C186" s="20">
         <v>1</v>
@@ -4348,7 +4369,7 @@
     </row>
     <row r="189" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B189" s="21" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C189" s="20">
         <v>1.2</v>
@@ -4356,7 +4377,7 @@
     </row>
     <row r="190" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B190" s="21" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C190" s="20">
         <v>2</v>
@@ -4364,7 +4385,7 @@
     </row>
     <row r="191" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B191" s="21" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C191" s="20">
         <v>1.2</v>
@@ -4372,7 +4393,7 @@
     </row>
     <row r="192" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B192" s="21" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C192" s="20">
         <v>1.5</v>
@@ -4380,7 +4401,7 @@
     </row>
     <row r="193" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B193" s="21" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C193" s="20">
         <v>1</v>
@@ -4388,7 +4409,7 @@
     </row>
     <row r="194" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B194" s="21" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C194" s="20">
         <v>2</v>
@@ -4396,7 +4417,7 @@
     </row>
     <row r="195" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B195" s="21" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C195" s="20">
         <v>1.5</v>
@@ -4404,7 +4425,7 @@
     </row>
     <row r="196" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B196" s="21" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C196" s="20">
         <v>1</v>
@@ -4412,7 +4433,7 @@
     </row>
     <row r="197" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B197" s="21" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C197" s="20">
         <v>1</v>
@@ -4428,7 +4449,7 @@
     </row>
     <row r="200" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B200" s="21" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C200" s="20">
         <v>1</v>
@@ -4436,7 +4457,7 @@
     </row>
     <row r="201" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B201" s="21" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C201" s="20">
         <v>1.2</v>
@@ -4444,7 +4465,7 @@
     </row>
     <row r="202" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B202" s="21" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C202" s="20">
         <v>1.5</v>
@@ -4452,7 +4473,7 @@
     </row>
     <row r="203" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B203" s="21" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C203" s="20">
         <v>1.2</v>
@@ -4460,7 +4481,7 @@
     </row>
     <row r="204" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B204" s="21" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C204" s="20">
         <v>1</v>
@@ -4468,7 +4489,7 @@
     </row>
     <row r="205" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B205" s="21" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C205" s="20">
         <v>0.8</v>
@@ -4476,7 +4497,7 @@
     </row>
     <row r="206" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B206" s="21" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C206" s="20">
         <v>1.5</v>
@@ -4484,7 +4505,7 @@
     </row>
     <row r="207" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B207" s="21" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C207" s="20">
         <v>1</v>
@@ -4492,7 +4513,7 @@
     </row>
     <row r="208" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B208" s="21" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C208" s="20">
         <v>1</v>
@@ -4500,7 +4521,7 @@
     </row>
     <row r="209" spans="1:5" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A209" s="24" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B209" s="21"/>
       <c r="C209" s="20"/>
@@ -4510,7 +4531,7 @@
     <row r="210" spans="1:5" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A210" s="24"/>
       <c r="B210" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C210" s="22">
         <v>1</v>
@@ -4521,7 +4542,7 @@
     <row r="211" spans="1:5" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A211" s="24"/>
       <c r="B211" s="22" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C211" s="22">
         <v>1</v>
@@ -4532,7 +4553,7 @@
     <row r="212" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A212" s="24"/>
       <c r="B212" s="22" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C212" s="22">
         <v>1.8</v>
@@ -4543,7 +4564,7 @@
     <row r="213" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A213" s="24"/>
       <c r="B213" s="22" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C213" s="22">
         <v>0.8</v>
@@ -4554,7 +4575,7 @@
     <row r="214" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A214" s="24"/>
       <c r="B214" s="22" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C214" s="22">
         <v>0.8</v>
@@ -4565,7 +4586,7 @@
     <row r="215" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A215" s="24"/>
       <c r="B215" s="22" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C215" s="22">
         <v>1.5</v>
@@ -4576,7 +4597,7 @@
     <row r="216" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A216" s="24"/>
       <c r="B216" s="22" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C216" s="22">
         <v>1</v>
@@ -4587,7 +4608,7 @@
     <row r="217" spans="1:5" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A217" s="24"/>
       <c r="B217" s="22" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="C217" s="22">
         <v>1</v>
@@ -4598,7 +4619,7 @@
     <row r="218" spans="1:5" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A218" s="24"/>
       <c r="B218" s="22" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C218" s="22">
         <v>0.7</v>
@@ -4609,7 +4630,7 @@
     <row r="219" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A219" s="24"/>
       <c r="B219" s="22" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C219" s="22">
         <v>0.6</v>
@@ -4620,7 +4641,7 @@
     <row r="220" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A220" s="24"/>
       <c r="B220" s="22" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C220" s="22">
         <v>0.6</v>
@@ -4630,7 +4651,7 @@
     </row>
     <row r="221" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A221" s="24" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B221" s="22"/>
       <c r="C221" s="22"/>
@@ -4640,7 +4661,7 @@
     <row r="222" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A222" s="24"/>
       <c r="B222" s="22" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C222" s="22">
         <v>1</v>
@@ -4651,7 +4672,7 @@
     <row r="223" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A223" s="24"/>
       <c r="B223" s="22" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="C223" s="22">
         <v>2</v>
@@ -4662,7 +4683,7 @@
     <row r="224" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A224" s="24"/>
       <c r="B224" s="22" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C224" s="22">
         <v>1.8</v>
@@ -4673,7 +4694,7 @@
     <row r="225" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A225" s="24"/>
       <c r="B225" s="22" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="C225" s="22">
         <v>1.8</v>
@@ -4684,7 +4705,7 @@
     <row r="226" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A226" s="24"/>
       <c r="B226" s="22" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C226" s="22">
         <v>1.2</v>
@@ -4695,7 +4716,7 @@
     <row r="227" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A227" s="24"/>
       <c r="B227" s="22" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C227" s="22">
         <v>2</v>
@@ -4706,7 +4727,7 @@
     <row r="228" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A228" s="24"/>
       <c r="B228" s="22" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C228" s="22">
         <v>1.2</v>
@@ -4717,7 +4738,7 @@
     <row r="229" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A229" s="24"/>
       <c r="B229" s="22" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C229" s="22">
         <v>1.2</v>
@@ -4728,7 +4749,7 @@
     <row r="230" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A230" s="24"/>
       <c r="B230" s="22" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="C230" s="22">
         <v>2</v>
@@ -4739,7 +4760,7 @@
     <row r="231" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A231" s="24"/>
       <c r="B231" s="22" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C231" s="22">
         <v>1</v>
@@ -4749,7 +4770,7 @@
     </row>
     <row r="232" spans="1:5" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A232" s="24" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B232" s="22"/>
       <c r="C232" s="22"/>
@@ -4759,7 +4780,7 @@
     <row r="233" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A233" s="24"/>
       <c r="B233" s="22" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="C233" s="22">
         <v>1</v>
@@ -4770,7 +4791,7 @@
     <row r="234" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A234" s="24"/>
       <c r="B234" s="22" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="C234" s="22">
         <v>1</v>
@@ -4781,7 +4802,7 @@
     <row r="235" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A235" s="24"/>
       <c r="B235" s="22" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="C235" s="22">
         <v>1.2</v>
@@ -4792,7 +4813,7 @@
     <row r="236" spans="1:5" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A236" s="24"/>
       <c r="B236" s="22" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="C236" s="22">
         <v>0.8</v>
@@ -4803,7 +4824,7 @@
     <row r="237" spans="1:5" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A237" s="24"/>
       <c r="B237" s="22" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="C237" s="22">
         <v>1</v>
@@ -4814,7 +4835,7 @@
     <row r="238" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A238" s="24"/>
       <c r="B238" s="22" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C238" s="22">
         <v>1.2</v>
@@ -4825,7 +4846,7 @@
     <row r="239" spans="1:5" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A239" s="24"/>
       <c r="B239" s="22" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C239" s="22">
         <v>0.8</v>
@@ -4835,7 +4856,7 @@
     </row>
     <row r="240" spans="1:5" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A240" s="24" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B240" s="22"/>
       <c r="C240" s="22"/>
@@ -4845,7 +4866,7 @@
     <row r="241" spans="1:5" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A241" s="24"/>
       <c r="B241" s="22" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C241" s="22">
         <v>0.8</v>
@@ -4856,7 +4877,7 @@
     <row r="242" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A242" s="24"/>
       <c r="B242" s="22" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="C242" s="22">
         <v>1.5</v>
@@ -4867,7 +4888,7 @@
     <row r="243" spans="1:5" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A243" s="24"/>
       <c r="B243" s="22" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="C243" s="22">
         <v>1</v>
@@ -4878,7 +4899,7 @@
     <row r="244" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A244" s="24"/>
       <c r="B244" s="22" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C244" s="22">
         <v>1.5</v>
@@ -4889,7 +4910,7 @@
     <row r="245" spans="1:5" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A245" s="24"/>
       <c r="B245" s="22" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C245" s="22">
         <v>1.2</v>
@@ -4899,7 +4920,7 @@
     </row>
     <row r="246" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B246" s="22" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C246" s="22">
         <v>1</v>
@@ -4913,7 +4934,7 @@
     </row>
     <row r="249" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="B249" s="21" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C249" s="20">
         <v>1.2</v>
@@ -4921,7 +4942,7 @@
     </row>
     <row r="250" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="B250" s="21" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C250" s="20">
         <v>1.5</v>
@@ -4929,7 +4950,7 @@
     </row>
     <row r="251" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B251" s="21" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C251" s="20">
         <v>1</v>
@@ -4937,7 +4958,7 @@
     </row>
     <row r="252" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B252" s="21" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C252" s="20">
         <v>2</v>
@@ -4945,7 +4966,7 @@
     </row>
     <row r="253" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B253" s="21" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C253" s="20">
         <v>1</v>
@@ -4953,7 +4974,7 @@
     </row>
     <row r="254" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B254" s="21" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C254" s="20">
         <v>1.5</v>
@@ -4961,7 +4982,7 @@
     </row>
     <row r="255" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="B255" s="21" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C255" s="20">
         <v>1</v>
@@ -4969,7 +4990,7 @@
     </row>
     <row r="256" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B256" s="21" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C256" s="20">
         <v>1</v>
@@ -4983,7 +5004,7 @@
     </row>
     <row r="259" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B259" s="21" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C259" s="20">
         <v>1.2</v>
@@ -4991,7 +5012,7 @@
     </row>
     <row r="260" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B260" s="21" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C260" s="20">
         <v>1</v>
@@ -4999,7 +5020,7 @@
     </row>
     <row r="261" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B261" s="21" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C261" s="20">
         <v>1.2</v>
@@ -5007,7 +5028,7 @@
     </row>
     <row r="262" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B262" s="21" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C262" s="20">
         <v>1.5</v>
@@ -5015,7 +5036,7 @@
     </row>
     <row r="263" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B263" s="21" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C263" s="20">
         <v>1.5</v>
@@ -5023,7 +5044,7 @@
     </row>
     <row r="264" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B264" s="21" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C264" s="20">
         <v>1</v>
@@ -5031,7 +5052,7 @@
     </row>
     <row r="265" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B265" s="21" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C265" s="20">
         <v>1</v>
@@ -5045,7 +5066,7 @@
     </row>
     <row r="268" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B268" s="21" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C268" s="20">
         <v>1.2</v>
@@ -5053,7 +5074,7 @@
     </row>
     <row r="269" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B269" s="21" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C269" s="20">
         <v>1</v>
@@ -5061,7 +5082,7 @@
     </row>
     <row r="270" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B270" s="21" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C270" s="20">
         <v>0.6</v>
@@ -5069,7 +5090,7 @@
     </row>
     <row r="271" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B271" s="21" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C271" s="20">
         <v>1.5</v>
@@ -5077,7 +5098,7 @@
     </row>
     <row r="272" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B272" s="21" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C272" s="20">
         <v>1.5</v>
@@ -5085,7 +5106,7 @@
     </row>
     <row r="273" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B273" s="21" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C273" s="20">
         <v>1.5</v>
@@ -5093,7 +5114,7 @@
     </row>
     <row r="274" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B274" s="21" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C274" s="20">
         <v>1</v>
@@ -5101,7 +5122,7 @@
     </row>
     <row r="275" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B275" s="21" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C275" s="20">
         <v>1</v>
@@ -5115,7 +5136,7 @@
     </row>
     <row r="278" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B278" s="21" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C278" s="20">
         <v>1</v>
@@ -5123,7 +5144,7 @@
     </row>
     <row r="279" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B279" s="21" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C279" s="20">
         <v>1.5</v>
@@ -5131,7 +5152,7 @@
     </row>
     <row r="280" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B280" s="21" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C280" s="20">
         <v>1.5</v>
@@ -5139,7 +5160,7 @@
     </row>
     <row r="281" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B281" s="21" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C281" s="20">
         <v>2</v>
@@ -5147,7 +5168,7 @@
     </row>
     <row r="282" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B282" s="21" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C282" s="20">
         <v>1.5</v>
@@ -5155,7 +5176,7 @@
     </row>
     <row r="283" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B283" s="21" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C283" s="20">
         <v>1</v>
@@ -5163,7 +5184,7 @@
     </row>
     <row r="284" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B284" s="21" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C284" s="20">
         <v>1.5</v>
@@ -5171,7 +5192,7 @@
     </row>
     <row r="285" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B285" s="21" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C285" s="20">
         <v>1</v>
@@ -5179,7 +5200,7 @@
     </row>
     <row r="286" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B286" s="21" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C286" s="20">
         <v>1</v>
@@ -5193,7 +5214,7 @@
     </row>
     <row r="289" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B289" s="21" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C289" s="20">
         <v>1.2</v>
@@ -5201,7 +5222,7 @@
     </row>
     <row r="290" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B290" s="21" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C290" s="20">
         <v>1.2</v>
@@ -5209,7 +5230,7 @@
     </row>
     <row r="291" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B291" s="21" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C291" s="20">
         <v>1.2</v>
@@ -5217,7 +5238,7 @@
     </row>
     <row r="292" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B292" s="21" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C292" s="20">
         <v>2</v>
@@ -5225,7 +5246,7 @@
     </row>
     <row r="293" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B293" s="21" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C293" s="20">
         <v>1.5</v>
@@ -5233,7 +5254,7 @@
     </row>
     <row r="294" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B294" s="21" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C294" s="20">
         <v>1</v>
@@ -5241,7 +5262,7 @@
     </row>
     <row r="295" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B295" s="21" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C295" s="20">
         <v>1</v>
@@ -5255,7 +5276,7 @@
     </row>
     <row r="298" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B298" s="21" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C298" s="20">
         <v>0.8</v>
@@ -5263,7 +5284,7 @@
     </row>
     <row r="299" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B299" s="21" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C299" s="20">
         <v>0.8</v>
@@ -5271,7 +5292,7 @@
     </row>
     <row r="300" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B300" s="21" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C300" s="20">
         <v>1</v>
@@ -5279,7 +5300,7 @@
     </row>
     <row r="301" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B301" s="21" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C301" s="20">
         <v>1.5</v>
@@ -5287,7 +5308,7 @@
     </row>
     <row r="302" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B302" s="21" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C302" s="20">
         <v>1.5</v>
@@ -5295,7 +5316,7 @@
     </row>
     <row r="303" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B303" s="21" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C303" s="20">
         <v>1</v>
@@ -5303,7 +5324,7 @@
     </row>
     <row r="304" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B304" s="21" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C304" s="20">
         <v>1</v>
@@ -5317,7 +5338,7 @@
     </row>
     <row r="307" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B307" s="21" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C307" s="20">
         <v>1</v>
@@ -5325,7 +5346,7 @@
     </row>
     <row r="308" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B308" s="21" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C308" s="20">
         <v>1.5</v>
@@ -5333,7 +5354,7 @@
     </row>
     <row r="309" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B309" s="21" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C309" s="20">
         <v>1</v>
@@ -5341,7 +5362,7 @@
     </row>
     <row r="310" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B310" s="21" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C310" s="20">
         <v>1</v>
@@ -5349,7 +5370,7 @@
     </row>
     <row r="311" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B311" s="21" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C311" s="20">
         <v>1.5</v>
@@ -5357,7 +5378,7 @@
     </row>
     <row r="312" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B312" s="21" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C312" s="20">
         <v>1</v>
@@ -5365,7 +5386,7 @@
     </row>
     <row r="313" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B313" s="21" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C313" s="20">
         <v>1</v>
@@ -5379,7 +5400,7 @@
     </row>
     <row r="316" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B316" s="21" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C316" s="20">
         <v>1.5</v>
@@ -5387,7 +5408,7 @@
     </row>
     <row r="317" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B317" s="21" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C317" s="20">
         <v>1.5</v>
@@ -5395,7 +5416,7 @@
     </row>
     <row r="318" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B318" s="21" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C318" s="20">
         <v>1.2</v>
@@ -5403,7 +5424,7 @@
     </row>
     <row r="319" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B319" s="21" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C319" s="20">
         <v>0.8</v>
@@ -5411,7 +5432,7 @@
     </row>
     <row r="320" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B320" s="21" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C320" s="20">
         <v>1</v>
@@ -5419,7 +5440,7 @@
     </row>
     <row r="321" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B321" s="21" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C321" s="20">
         <v>1</v>
@@ -5433,7 +5454,7 @@
     </row>
     <row r="324" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B324" s="21" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C324" s="20">
         <v>1</v>
@@ -5441,7 +5462,7 @@
     </row>
     <row r="325" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B325" s="21" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C325" s="20">
         <v>1.2</v>
@@ -5449,7 +5470,7 @@
     </row>
     <row r="326" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B326" s="21" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C326" s="20">
         <v>0.8</v>
@@ -5457,7 +5478,7 @@
     </row>
     <row r="327" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B327" s="21" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C327" s="20">
         <v>0.8</v>
@@ -5465,7 +5486,7 @@
     </row>
     <row r="328" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B328" s="21" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C328" s="20">
         <v>1.5</v>
@@ -5473,7 +5494,7 @@
     </row>
     <row r="329" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B329" s="21" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C329" s="20">
         <v>1</v>
@@ -5481,7 +5502,7 @@
     </row>
     <row r="330" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B330" s="21" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C330" s="20">
         <v>1</v>
@@ -5495,7 +5516,7 @@
     </row>
     <row r="333" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B333" s="21" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C333" s="20">
         <v>1.2</v>
@@ -5503,7 +5524,7 @@
     </row>
     <row r="334" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B334" s="21" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C334" s="20">
         <v>1</v>
@@ -5511,7 +5532,7 @@
     </row>
     <row r="335" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B335" s="21" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C335" s="20">
         <v>1</v>
@@ -5519,7 +5540,7 @@
     </row>
     <row r="336" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B336" s="21" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C336" s="20">
         <v>1.2</v>
@@ -5527,7 +5548,7 @@
     </row>
     <row r="337" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B337" s="21" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C337" s="20">
         <v>1.5</v>
@@ -5535,7 +5556,7 @@
     </row>
     <row r="338" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="B338" s="21" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C338" s="20">
         <v>1</v>
@@ -5543,7 +5564,7 @@
     </row>
     <row r="339" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B339" s="21" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C339" s="20">
         <v>1</v>
@@ -5557,7 +5578,7 @@
     </row>
     <row r="342" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B342" s="21" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C342" s="20">
         <v>1.2</v>
@@ -5565,7 +5586,7 @@
     </row>
     <row r="343" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="B343" s="21" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C343" s="20">
         <v>1.2</v>
@@ -5573,7 +5594,7 @@
     </row>
     <row r="344" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="B344" s="21" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C344" s="20">
         <v>1.5</v>
@@ -5581,7 +5602,7 @@
     </row>
     <row r="345" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B345" s="21" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C345" s="20">
         <v>0.8</v>
@@ -5589,7 +5610,7 @@
     </row>
     <row r="346" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B346" s="21" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C346" s="20">
         <v>1</v>
@@ -5597,7 +5618,7 @@
     </row>
     <row r="347" spans="1:5" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A347" s="24" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B347" s="21"/>
       <c r="C347" s="20"/>
@@ -5607,7 +5628,7 @@
     <row r="348" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A348" s="24"/>
       <c r="B348" s="22" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C348" s="22">
         <v>0.8</v>
@@ -5618,7 +5639,7 @@
     <row r="349" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A349" s="24"/>
       <c r="B349" s="22" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="C349" s="22">
         <v>0.8</v>
@@ -5629,7 +5650,7 @@
     <row r="350" spans="1:5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A350" s="24"/>
       <c r="B350" s="22" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="C350" s="22">
         <v>0.8</v>
@@ -5639,7 +5660,7 @@
     </row>
     <row r="351" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="B351" s="22" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C351" s="22">
         <v>0.8</v>
@@ -5653,7 +5674,7 @@
     </row>
     <row r="354" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B354" s="21" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C354" s="20">
         <v>1.5</v>
@@ -5661,7 +5682,7 @@
     </row>
     <row r="355" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B355" s="21" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C355" s="20">
         <v>1.2</v>
@@ -5669,7 +5690,7 @@
     </row>
     <row r="356" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B356" s="21" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C356" s="20">
         <v>1.2</v>
@@ -5677,7 +5698,7 @@
     </row>
     <row r="357" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B357" s="21" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C357" s="20">
         <v>2</v>
@@ -5685,7 +5706,7 @@
     </row>
     <row r="358" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B358" s="21" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C358" s="20">
         <v>1.2</v>
@@ -5693,7 +5714,7 @@
     </row>
     <row r="359" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B359" s="21" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C359" s="20">
         <v>1.8</v>
@@ -5701,7 +5722,7 @@
     </row>
     <row r="360" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B360" s="21" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C360" s="20">
         <v>1.5</v>
@@ -5709,7 +5730,7 @@
     </row>
     <row r="361" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B361" s="21" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C361" s="20">
         <v>2</v>
@@ -5717,7 +5738,7 @@
     </row>
     <row r="362" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B362" s="21" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C362" s="20">
         <v>1</v>
@@ -5725,7 +5746,7 @@
     </row>
     <row r="363" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B363" s="21" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C363" s="20">
         <v>1</v>
@@ -5739,7 +5760,7 @@
     </row>
     <row r="366" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B366" s="21" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C366" s="20">
         <v>2</v>
@@ -5747,7 +5768,7 @@
     </row>
     <row r="367" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B367" s="21" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="C367" s="20">
         <v>1.2</v>
@@ -5755,7 +5776,7 @@
     </row>
     <row r="368" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B368" s="21" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C368" s="20">
         <v>3</v>
@@ -5763,7 +5784,7 @@
     </row>
     <row r="369" spans="2:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B369" s="21" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C369" s="20">
         <v>2.5</v>
@@ -5771,7 +5792,7 @@
     </row>
     <row r="370" spans="2:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B370" s="21" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C370" s="20">
         <v>1.5</v>
@@ -5779,7 +5800,7 @@
     </row>
     <row r="371" spans="2:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B371" s="21" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C371" s="20">
         <v>1</v>
@@ -5787,7 +5808,7 @@
     </row>
     <row r="372" spans="2:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B372" s="21" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C372" s="20">
         <v>1</v>

</xml_diff>